<commit_message>
Add DOCX/PDF for all 40 XLSX files, fix xlsx formatting with freeze panes
- Generate .docx and .pdf for all 40 xlsx files (employment_xlsx/ + root)
- Add convert_xlsx_to_docx_pdf.py script for xlsx→docx and xlsx→pdf conversion
- Fix xlsx formatting: add freeze panes, auto-filters, proper print setup
- Regenerate all xlsx files with improved structure
- Generate CODEBASE_SUMMARY.docx and CODEBASE_SUMMARY.pdf
- Update generate_employment_xlsx.py and generate_business_xlsx.py

https://claude.ai/code/session_014AKpynNrHyqLfWAM6MLBvL
</commit_message>
<xml_diff>
--- a/employment_xlsx/PECH_API_DEVELOPER_AGREEMENT.xlsx
+++ b/employment_xlsx/PECH_API_DEVELOPER_AGREEMENT.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,34 +59,6 @@
       <i val="1"/>
       <color rgb="00999999"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="000099CC"/>
-      <sz val="18"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <i val="1"/>
-      <color rgb="00F5A623"/>
-      <sz val="9"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="00888888"/>
-      <sz val="7"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <b val="1"/>
-      <color rgb="00E8F4F8"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="00AAAAAA"/>
-      <sz val="7"/>
     </font>
   </fonts>
   <fills count="8">
@@ -159,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -186,21 +158,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -275,36 +232,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1905000" cy="628650"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -596,7 +523,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N45"/>
+  <dimension ref="A1:N33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -615,31 +542,63 @@
     <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="40" customHeight="1">
-      <c r="A1" s="14" t="inlineStr">
+    <row r="1" ht="6" customHeight="1">
+      <c r="A1" s="1" t="inlineStr"/>
+      <c r="B1" s="1" t="inlineStr"/>
+      <c r="C1" s="1" t="inlineStr"/>
+      <c r="D1" s="1" t="inlineStr"/>
+      <c r="E1" s="1" t="inlineStr"/>
+      <c r="F1" s="1" t="inlineStr"/>
+      <c r="G1" s="1" t="inlineStr"/>
+      <c r="H1" s="1" t="inlineStr"/>
+      <c r="I1" s="1" t="inlineStr"/>
+      <c r="J1" s="1" t="inlineStr"/>
+      <c r="K1" s="1" t="inlineStr"/>
+      <c r="L1" s="1" t="inlineStr"/>
+      <c r="M1" s="1" t="inlineStr"/>
+      <c r="N1" s="1" t="inlineStr"/>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>PECH GROUP HOLDINGS LTD</t>
         </is>
       </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="15" t="inlineStr">
-        <is>
-          <t>Technology &amp; Infrastructure Enablers for People</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="4" customHeight="1">
-      <c r="A3" s="1" t="n"/>
-      <c r="B3" s="1" t="n"/>
-      <c r="C3" s="1" t="n"/>
-      <c r="D3" s="1" t="n"/>
-      <c r="E3" s="1" t="n"/>
-      <c r="F3" s="1" t="n"/>
-      <c r="G3" s="1" t="n"/>
-      <c r="H3" s="1" t="n"/>
-    </row>
-    <row r="4" ht="2" customHeight="1">
+      <c r="B2" s="3" t="n"/>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="3" t="n"/>
+      <c r="F2" s="3" t="n"/>
+      <c r="G2" s="3" t="n"/>
+      <c r="H2" s="3" t="n"/>
+      <c r="I2" s="3" t="n"/>
+      <c r="J2" s="3" t="n"/>
+      <c r="K2" s="3" t="n"/>
+      <c r="L2" s="3" t="n"/>
+      <c r="M2" s="3" t="n"/>
+      <c r="N2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>API DEVELOPER AGREEMENT TRACKER</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
+      <c r="M3" s="3" t="n"/>
+      <c r="N3" s="3" t="n"/>
+    </row>
+    <row r="4" ht="4" customHeight="1">
       <c r="A4" s="5" t="n"/>
       <c r="B4" s="5" t="n"/>
       <c r="C4" s="5" t="n"/>
@@ -648,167 +607,253 @@
       <c r="F4" s="5" t="n"/>
       <c r="G4" s="5" t="n"/>
       <c r="H4" s="5" t="n"/>
-    </row>
-    <row r="5" ht="16" customHeight="1">
-      <c r="A5" s="16" t="inlineStr">
-        <is>
-          <t>Lagos, Nigeria  |  pechgroupholdings.tech  |  Confidential</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="8" customHeight="1"/>
-    <row r="7" ht="8" customHeight="1">
-      <c r="A7" s="1" t="inlineStr"/>
-      <c r="B7" s="1" t="inlineStr"/>
-      <c r="C7" s="1" t="inlineStr"/>
-      <c r="D7" s="1" t="inlineStr"/>
-      <c r="E7" s="1" t="inlineStr"/>
-      <c r="F7" s="1" t="inlineStr"/>
-      <c r="G7" s="1" t="inlineStr"/>
-      <c r="H7" s="1" t="inlineStr"/>
-      <c r="I7" s="1" t="inlineStr"/>
-      <c r="J7" s="1" t="inlineStr"/>
-      <c r="K7" s="1" t="inlineStr"/>
-      <c r="L7" s="1" t="inlineStr"/>
-      <c r="M7" s="1" t="inlineStr"/>
-      <c r="N7" s="1" t="inlineStr"/>
-    </row>
+      <c r="I4" s="5" t="n"/>
+      <c r="J4" s="5" t="n"/>
+      <c r="K4" s="5" t="n"/>
+      <c r="L4" s="5" t="n"/>
+      <c r="M4" s="5" t="n"/>
+      <c r="N4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Lagos, Nigeria  |  pechgroupholdings.tech  |  Track external API developers  |  CONFIDENTIAL</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+      <c r="M5" s="3" t="n"/>
+      <c r="N5" s="3" t="n"/>
+    </row>
+    <row r="6" ht="4" customHeight="1">
+      <c r="A6" s="5" t="n"/>
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="5" t="n"/>
+      <c r="D6" s="5" t="n"/>
+      <c r="E6" s="5" t="n"/>
+      <c r="F6" s="5" t="n"/>
+      <c r="G6" s="5" t="n"/>
+      <c r="H6" s="1" t="n"/>
+      <c r="I6" s="1" t="n"/>
+      <c r="J6" s="1" t="n"/>
+      <c r="K6" s="1" t="n"/>
+      <c r="L6" s="1" t="n"/>
+      <c r="M6" s="1" t="n"/>
+      <c r="N6" s="1" t="n"/>
+    </row>
+    <row r="7" ht="8" customHeight="1"/>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>PECH GROUP HOLDINGS LTD</t>
-        </is>
-      </c>
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  API DEVELOPER REGISTER</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n"/>
+      <c r="C8" s="8" t="n"/>
+      <c r="D8" s="8" t="n"/>
+      <c r="E8" s="8" t="n"/>
+      <c r="F8" s="8" t="n"/>
+      <c r="G8" s="8" t="n"/>
+      <c r="H8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8" t="n"/>
+      <c r="K8" s="8" t="n"/>
+      <c r="L8" s="8" t="n"/>
+      <c r="M8" s="8" t="n"/>
+      <c r="N8" s="8" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>API DEVELOPER AGREEMENT TRACKER</t>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>Developer Name/Company</t>
+        </is>
+      </c>
+      <c r="C9" s="9" t="inlineStr">
+        <is>
+          <t>Contact Email</t>
+        </is>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>API Key Issued</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>End Date</t>
+        </is>
+      </c>
+      <c r="G9" s="9" t="inlineStr">
+        <is>
+          <t>API Access Tier</t>
+        </is>
+      </c>
+      <c r="H9" s="9" t="inlineStr">
+        <is>
+          <t>Rate Limit</t>
+        </is>
+      </c>
+      <c r="I9" s="9" t="inlineStr">
+        <is>
+          <t>Sandbox Access</t>
+        </is>
+      </c>
+      <c r="J9" s="9" t="inlineStr">
+        <is>
+          <t>Production Access</t>
+        </is>
+      </c>
+      <c r="K9" s="9" t="inlineStr">
+        <is>
+          <t>NDA Signed</t>
+        </is>
+      </c>
+      <c r="L9" s="9" t="inlineStr">
+        <is>
+          <t>Data Compliant</t>
+        </is>
+      </c>
+      <c r="M9" s="9" t="inlineStr">
+        <is>
+          <t>Agreement Ref.</t>
+        </is>
+      </c>
+      <c r="N9" s="9" t="inlineStr">
+        <is>
+          <t>Status</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="n"/>
-      <c r="B10" s="5" t="n"/>
-      <c r="C10" s="5" t="n"/>
-      <c r="D10" s="5" t="n"/>
-      <c r="E10" s="5" t="n"/>
-      <c r="F10" s="5" t="n"/>
-      <c r="G10" s="5" t="n"/>
-      <c r="H10" s="5" t="n"/>
-      <c r="I10" s="5" t="n"/>
-      <c r="J10" s="5" t="n"/>
-      <c r="K10" s="5" t="n"/>
-      <c r="L10" s="5" t="n"/>
-      <c r="M10" s="5" t="n"/>
-      <c r="N10" s="5" t="n"/>
+      <c r="A10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B10" s="10" t="n"/>
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="10" t="n"/>
+      <c r="H10" s="10" t="n"/>
+      <c r="I10" s="10" t="n"/>
+      <c r="J10" s="10" t="n"/>
+      <c r="K10" s="10" t="n"/>
+      <c r="L10" s="10" t="n"/>
+      <c r="M10" s="10" t="n"/>
+      <c r="N10" s="10" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Lagos, Nigeria  |  pechgroupholdings.tech  |  Track external API developers  |  CONFIDENTIAL</t>
-        </is>
-      </c>
+      <c r="A11" s="11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" s="11" t="n"/>
+      <c r="C11" s="11" t="n"/>
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
+      <c r="J11" s="11" t="n"/>
+      <c r="K11" s="11" t="n"/>
+      <c r="L11" s="11" t="n"/>
+      <c r="M11" s="11" t="n"/>
+      <c r="N11" s="11" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="n"/>
-      <c r="B12" s="5" t="n"/>
-      <c r="C12" s="5" t="n"/>
-      <c r="D12" s="5" t="n"/>
-      <c r="E12" s="5" t="n"/>
-      <c r="F12" s="5" t="n"/>
-      <c r="G12" s="5" t="n"/>
-      <c r="H12" s="1" t="n"/>
-      <c r="I12" s="1" t="n"/>
-      <c r="J12" s="1" t="n"/>
-      <c r="K12" s="1" t="n"/>
-      <c r="L12" s="1" t="n"/>
-      <c r="M12" s="1" t="n"/>
-      <c r="N12" s="1" t="n"/>
-    </row>
-    <row r="13"/>
+      <c r="A12" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B12" s="10" t="n"/>
+      <c r="C12" s="10" t="n"/>
+      <c r="D12" s="10" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="10" t="n"/>
+      <c r="I12" s="10" t="n"/>
+      <c r="J12" s="10" t="n"/>
+      <c r="K12" s="10" t="n"/>
+      <c r="L12" s="10" t="n"/>
+      <c r="M12" s="10" t="n"/>
+      <c r="N12" s="10" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B13" s="11" t="n"/>
+      <c r="C13" s="11" t="n"/>
+      <c r="D13" s="11" t="n"/>
+      <c r="E13" s="11" t="n"/>
+      <c r="F13" s="11" t="n"/>
+      <c r="G13" s="11" t="n"/>
+      <c r="H13" s="11" t="n"/>
+      <c r="I13" s="11" t="n"/>
+      <c r="J13" s="11" t="n"/>
+      <c r="K13" s="11" t="n"/>
+      <c r="L13" s="11" t="n"/>
+      <c r="M13" s="11" t="n"/>
+      <c r="N13" s="11" t="n"/>
+    </row>
     <row r="14">
-      <c r="A14" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  API DEVELOPER REGISTER</t>
-        </is>
-      </c>
+      <c r="A14" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
+      <c r="G14" s="10" t="n"/>
+      <c r="H14" s="10" t="n"/>
+      <c r="I14" s="10" t="n"/>
+      <c r="J14" s="10" t="n"/>
+      <c r="K14" s="10" t="n"/>
+      <c r="L14" s="10" t="n"/>
+      <c r="M14" s="10" t="n"/>
+      <c r="N14" s="10" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="9" t="inlineStr">
-        <is>
-          <t>#</t>
-        </is>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>Developer Name/Company</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>Contact Email</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>API Key Issued</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="G15" s="9" t="inlineStr">
-        <is>
-          <t>API Access Tier</t>
-        </is>
-      </c>
-      <c r="H15" s="9" t="inlineStr">
-        <is>
-          <t>Rate Limit</t>
-        </is>
-      </c>
-      <c r="I15" s="9" t="inlineStr">
-        <is>
-          <t>Sandbox Access</t>
-        </is>
-      </c>
-      <c r="J15" s="9" t="inlineStr">
-        <is>
-          <t>Production Access</t>
-        </is>
-      </c>
-      <c r="K15" s="9" t="inlineStr">
-        <is>
-          <t>NDA Signed</t>
-        </is>
-      </c>
-      <c r="L15" s="9" t="inlineStr">
-        <is>
-          <t>Data Compliant</t>
-        </is>
-      </c>
-      <c r="M15" s="9" t="inlineStr">
-        <is>
-          <t>Agreement Ref.</t>
-        </is>
-      </c>
-      <c r="N15" s="9" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
+      <c r="A15" s="11" t="n">
+        <v>6</v>
+      </c>
+      <c r="B15" s="11" t="n"/>
+      <c r="C15" s="11" t="n"/>
+      <c r="D15" s="11" t="n"/>
+      <c r="E15" s="11" t="n"/>
+      <c r="F15" s="11" t="n"/>
+      <c r="G15" s="11" t="n"/>
+      <c r="H15" s="11" t="n"/>
+      <c r="I15" s="11" t="n"/>
+      <c r="J15" s="11" t="n"/>
+      <c r="K15" s="11" t="n"/>
+      <c r="L15" s="11" t="n"/>
+      <c r="M15" s="11" t="n"/>
+      <c r="N15" s="11" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="10" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="B16" s="10" t="n"/>
       <c r="C16" s="10" t="n"/>
@@ -826,7 +871,7 @@
     </row>
     <row r="17">
       <c r="A17" s="11" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="B17" s="11" t="n"/>
       <c r="C17" s="11" t="n"/>
@@ -844,7 +889,7 @@
     </row>
     <row r="18">
       <c r="A18" s="10" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="B18" s="10" t="n"/>
       <c r="C18" s="10" t="n"/>
@@ -862,7 +907,7 @@
     </row>
     <row r="19">
       <c r="A19" s="11" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="B19" s="11" t="n"/>
       <c r="C19" s="11" t="n"/>
@@ -880,7 +925,7 @@
     </row>
     <row r="20">
       <c r="A20" s="10" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="B20" s="10" t="n"/>
       <c r="C20" s="10" t="n"/>
@@ -898,7 +943,7 @@
     </row>
     <row r="21">
       <c r="A21" s="11" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="B21" s="11" t="n"/>
       <c r="C21" s="11" t="n"/>
@@ -916,7 +961,7 @@
     </row>
     <row r="22">
       <c r="A22" s="10" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="B22" s="10" t="n"/>
       <c r="C22" s="10" t="n"/>
@@ -934,7 +979,7 @@
     </row>
     <row r="23">
       <c r="A23" s="11" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="B23" s="11" t="n"/>
       <c r="C23" s="11" t="n"/>
@@ -952,7 +997,7 @@
     </row>
     <row r="24">
       <c r="A24" s="10" t="n">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B24" s="10" t="n"/>
       <c r="C24" s="10" t="n"/>
@@ -970,7 +1015,7 @@
     </row>
     <row r="25">
       <c r="A25" s="11" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="B25" s="11" t="n"/>
       <c r="C25" s="11" t="n"/>
@@ -988,7 +1033,7 @@
     </row>
     <row r="26">
       <c r="A26" s="10" t="n">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B26" s="10" t="n"/>
       <c r="C26" s="10" t="n"/>
@@ -1006,7 +1051,7 @@
     </row>
     <row r="27">
       <c r="A27" s="11" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="B27" s="11" t="n"/>
       <c r="C27" s="11" t="n"/>
@@ -1024,7 +1069,7 @@
     </row>
     <row r="28">
       <c r="A28" s="10" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B28" s="10" t="n"/>
       <c r="C28" s="10" t="n"/>
@@ -1042,7 +1087,7 @@
     </row>
     <row r="29">
       <c r="A29" s="11" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="B29" s="11" t="n"/>
       <c r="C29" s="11" t="n"/>
@@ -1058,202 +1103,63 @@
       <c r="M29" s="11" t="n"/>
       <c r="N29" s="11" t="n"/>
     </row>
-    <row r="30">
-      <c r="A30" s="10" t="n">
-        <v>15</v>
-      </c>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
-      <c r="H30" s="10" t="n"/>
-      <c r="I30" s="10" t="n"/>
-      <c r="J30" s="10" t="n"/>
-      <c r="K30" s="10" t="n"/>
-      <c r="L30" s="10" t="n"/>
-      <c r="M30" s="10" t="n"/>
-      <c r="N30" s="10" t="n"/>
-    </row>
     <row r="31" ht="3" customHeight="1">
-      <c r="A31" s="11" t="n">
-        <v>16</v>
-      </c>
-      <c r="B31" s="11" t="n"/>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="11" t="n"/>
-      <c r="E31" s="11" t="n"/>
-      <c r="F31" s="11" t="n"/>
-      <c r="G31" s="11" t="n"/>
-      <c r="H31" s="11" t="n"/>
-      <c r="I31" s="11" t="n"/>
-      <c r="J31" s="11" t="n"/>
-      <c r="K31" s="11" t="n"/>
-      <c r="L31" s="11" t="n"/>
-      <c r="M31" s="11" t="n"/>
-      <c r="N31" s="11" t="n"/>
+      <c r="A31" s="5" t="n"/>
+      <c r="B31" s="5" t="n"/>
+      <c r="C31" s="5" t="n"/>
+      <c r="D31" s="5" t="n"/>
+      <c r="E31" s="5" t="n"/>
+      <c r="F31" s="5" t="n"/>
+      <c r="G31" s="5" t="n"/>
+      <c r="H31" s="5" t="n"/>
+      <c r="I31" s="5" t="n"/>
+      <c r="J31" s="5" t="n"/>
+      <c r="K31" s="5" t="n"/>
+      <c r="L31" s="5" t="n"/>
+      <c r="M31" s="5" t="n"/>
+      <c r="N31" s="5" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="10" t="n">
-        <v>17</v>
-      </c>
-      <c r="B32" s="10" t="n"/>
-      <c r="C32" s="10" t="n"/>
-      <c r="D32" s="10" t="n"/>
-      <c r="E32" s="10" t="n"/>
-      <c r="F32" s="10" t="n"/>
-      <c r="G32" s="10" t="n"/>
-      <c r="H32" s="10" t="n"/>
-      <c r="I32" s="10" t="n"/>
-      <c r="J32" s="10" t="n"/>
-      <c r="K32" s="10" t="n"/>
-      <c r="L32" s="10" t="n"/>
-      <c r="M32" s="10" t="n"/>
-      <c r="N32" s="10" t="n"/>
+      <c r="A32" s="12" t="inlineStr">
+        <is>
+          <t>PECH Group Holdings Ltd  |  Confidential  |  pechgroupholdings.tech  |  Technology &amp; Infrastructure Enablers for People</t>
+        </is>
+      </c>
+      <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
+      <c r="E32" s="13" t="n"/>
+      <c r="F32" s="13" t="n"/>
+      <c r="G32" s="13" t="n"/>
+      <c r="H32" s="13" t="n"/>
+      <c r="I32" s="13" t="n"/>
+      <c r="J32" s="13" t="n"/>
+      <c r="K32" s="13" t="n"/>
+      <c r="L32" s="13" t="n"/>
+      <c r="M32" s="13" t="n"/>
+      <c r="N32" s="13" t="n"/>
     </row>
     <row r="33" ht="3" customHeight="1">
-      <c r="A33" s="11" t="n">
-        <v>18</v>
-      </c>
-      <c r="B33" s="11" t="n"/>
-      <c r="C33" s="11" t="n"/>
-      <c r="D33" s="11" t="n"/>
-      <c r="E33" s="11" t="n"/>
-      <c r="F33" s="11" t="n"/>
-      <c r="G33" s="11" t="n"/>
-      <c r="H33" s="11" t="n"/>
-      <c r="I33" s="11" t="n"/>
-      <c r="J33" s="11" t="n"/>
-      <c r="K33" s="11" t="n"/>
-      <c r="L33" s="11" t="n"/>
-      <c r="M33" s="11" t="n"/>
-      <c r="N33" s="11" t="n"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="B34" s="10" t="n"/>
-      <c r="C34" s="10" t="n"/>
-      <c r="D34" s="10" t="n"/>
-      <c r="E34" s="10" t="n"/>
-      <c r="F34" s="10" t="n"/>
-      <c r="G34" s="10" t="n"/>
-      <c r="H34" s="10" t="n"/>
-      <c r="I34" s="10" t="n"/>
-      <c r="J34" s="10" t="n"/>
-      <c r="K34" s="10" t="n"/>
-      <c r="L34" s="10" t="n"/>
-      <c r="M34" s="10" t="n"/>
-      <c r="N34" s="10" t="n"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="11" t="n">
-        <v>20</v>
-      </c>
-      <c r="B35" s="11" t="n"/>
-      <c r="C35" s="11" t="n"/>
-      <c r="D35" s="11" t="n"/>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="11" t="n"/>
-      <c r="G35" s="11" t="n"/>
-      <c r="H35" s="11" t="n"/>
-      <c r="I35" s="11" t="n"/>
-      <c r="J35" s="11" t="n"/>
-      <c r="K35" s="11" t="n"/>
-      <c r="L35" s="11" t="n"/>
-      <c r="M35" s="11" t="n"/>
-      <c r="N35" s="11" t="n"/>
-    </row>
-    <row r="36"/>
-    <row r="37">
-      <c r="A37" s="5" t="n"/>
-      <c r="B37" s="5" t="n"/>
-      <c r="C37" s="5" t="n"/>
-      <c r="D37" s="5" t="n"/>
-      <c r="E37" s="5" t="n"/>
-      <c r="F37" s="5" t="n"/>
-      <c r="G37" s="5" t="n"/>
-      <c r="H37" s="5" t="n"/>
-      <c r="I37" s="5" t="n"/>
-      <c r="J37" s="5" t="n"/>
-      <c r="K37" s="5" t="n"/>
-      <c r="L37" s="5" t="n"/>
-      <c r="M37" s="5" t="n"/>
-      <c r="N37" s="5" t="n"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>PECH Group Holdings Ltd  |  Confidential  |  pechgroupholdings.tech  |  Technology &amp; Infrastructure Enablers for People</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="n"/>
-      <c r="B39" s="1" t="n"/>
-      <c r="C39" s="1" t="n"/>
-      <c r="D39" s="1" t="n"/>
-      <c r="E39" s="1" t="n"/>
-      <c r="F39" s="1" t="n"/>
-      <c r="G39" s="1" t="n"/>
-      <c r="H39" s="1" t="n"/>
-      <c r="I39" s="1" t="n"/>
-      <c r="J39" s="1" t="n"/>
-      <c r="K39" s="1" t="n"/>
-      <c r="L39" s="1" t="n"/>
-      <c r="M39" s="1" t="n"/>
-      <c r="N39" s="1" t="n"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="17" t="inlineStr">
-        <is>
-          <t>PECH GROUP HOLDINGS LTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" s="17" t="inlineStr">
-        <is>
-          <t>PECH GROUP HOLDINGS LTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
-        <is>
-          <t>PECH GROUP HOLDINGS LTD</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" s="18" t="inlineStr">
-        <is>
-          <t>Confidential — PECH Group Holdings Ltd — Lagos, Nigeria — pechgroupholdings.tech</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" s="1" t="n"/>
-      <c r="B45" s="1" t="n"/>
-      <c r="C45" s="1" t="n"/>
-      <c r="D45" s="1" t="n"/>
-      <c r="E45" s="1" t="n"/>
-      <c r="F45" s="1" t="n"/>
-      <c r="G45" s="1" t="n"/>
-      <c r="H45" s="1" t="n"/>
+      <c r="A33" s="1" t="n"/>
+      <c r="B33" s="1" t="n"/>
+      <c r="C33" s="1" t="n"/>
+      <c r="D33" s="1" t="n"/>
+      <c r="E33" s="1" t="n"/>
+      <c r="F33" s="1" t="n"/>
+      <c r="G33" s="1" t="n"/>
+      <c r="H33" s="1" t="n"/>
+      <c r="I33" s="1" t="n"/>
+      <c r="J33" s="1" t="n"/>
+      <c r="K33" s="1" t="n"/>
+      <c r="L33" s="1" t="n"/>
+      <c r="M33" s="1" t="n"/>
+      <c r="N33" s="1" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="5">
     <mergeCell ref="A8:N8"/>
     <mergeCell ref="A3:N3"/>
-    <mergeCell ref="A43:H43"/>
     <mergeCell ref="A2:N2"/>
-    <mergeCell ref="A42:H42"/>
-    <mergeCell ref="A41:H41"/>
-    <mergeCell ref="A44:H44"/>
-    <mergeCell ref="A1:H1"/>
     <mergeCell ref="A5:N5"/>
     <mergeCell ref="A32:N32"/>
   </mergeCells>
@@ -1266,15 +1172,6 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader>&amp;C&amp;8 PECH Group Holdings Ltd | Confidential</oddHeader>
-    <oddFooter>&amp;C&amp;7 PECH Group Holdings Ltd | Lagos, Nigeria | pechgroupholdings.tech</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix xlsx layout/formatting: explicit row heights, alignment, zoom, gridlines off, footer cleanup
- Set explicit row height (22px) on all data rows to prevent inconsistent sizing
- Add cell.alignment = ALIGN_LEFT to all data cells for consistent text positioning
- Set zoom to 100% and hide gridlines for cleaner appearance with explicit borders
- Remove duplicate "PECH Group Holdings Ltd" from footer text
- Add no_border styling to header/footer decorative rows to prevent grid artifacts
- Fill spacer row (row 7) with white + no border for clean separation
- Fix scoring rubric using wrong worksheet reference (ws vs ws2)
- All 39 xlsx files regenerated with fixes

https://claude.ai/code/session_014AKpynNrHyqLfWAM6MLBvL
</commit_message>
<xml_diff>
--- a/employment_xlsx/PECH_API_DEVELOPER_AGREEMENT.xlsx
+++ b/employment_xlsx/PECH_API_DEVELOPER_AGREEMENT.xlsx
@@ -88,14 +88,14 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000099CC"/>
-        <bgColor rgb="000099CC"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
+        <fgColor rgb="000099CC"/>
+        <bgColor rgb="000099CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,13 +105,19 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
     </border>
     <border>
       <left style="thin">
@@ -133,31 +139,35 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -650,458 +660,473 @@
       <c r="M6" s="1" t="n"/>
       <c r="N6" s="1" t="n"/>
     </row>
-    <row r="7" ht="8" customHeight="1"/>
+    <row r="7" ht="8" customHeight="1">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="7" t="n"/>
+      <c r="I7" s="7" t="n"/>
+      <c r="J7" s="7" t="n"/>
+      <c r="K7" s="7" t="n"/>
+      <c r="L7" s="7" t="n"/>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="7" t="n"/>
+    </row>
     <row r="8" ht="26" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">  API DEVELOPER REGISTER</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8" t="n"/>
-      <c r="K8" s="8" t="n"/>
-      <c r="L8" s="8" t="n"/>
-      <c r="M8" s="8" t="n"/>
-      <c r="N8" s="8" t="n"/>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9" t="n"/>
+      <c r="D8" s="9" t="n"/>
+      <c r="E8" s="9" t="n"/>
+      <c r="F8" s="9" t="n"/>
+      <c r="G8" s="9" t="n"/>
+      <c r="H8" s="9" t="n"/>
+      <c r="I8" s="9" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="9" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="n"/>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="A9" s="9" t="inlineStr">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>#</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="10" t="inlineStr">
         <is>
           <t>Developer Name/Company</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="10" t="inlineStr">
         <is>
           <t>Contact Email</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
+      <c r="D9" s="10" t="inlineStr">
         <is>
           <t>API Key Issued</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>Start Date</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
+      <c r="F9" s="10" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="G9" s="9" t="inlineStr">
+      <c r="G9" s="10" t="inlineStr">
         <is>
           <t>API Access Tier</t>
         </is>
       </c>
-      <c r="H9" s="9" t="inlineStr">
+      <c r="H9" s="10" t="inlineStr">
         <is>
           <t>Rate Limit</t>
         </is>
       </c>
-      <c r="I9" s="9" t="inlineStr">
+      <c r="I9" s="10" t="inlineStr">
         <is>
           <t>Sandbox Access</t>
         </is>
       </c>
-      <c r="J9" s="9" t="inlineStr">
+      <c r="J9" s="10" t="inlineStr">
         <is>
           <t>Production Access</t>
         </is>
       </c>
-      <c r="K9" s="9" t="inlineStr">
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>NDA Signed</t>
         </is>
       </c>
-      <c r="L9" s="9" t="inlineStr">
+      <c r="L9" s="10" t="inlineStr">
         <is>
           <t>Data Compliant</t>
         </is>
       </c>
-      <c r="M9" s="9" t="inlineStr">
+      <c r="M9" s="10" t="inlineStr">
         <is>
           <t>Agreement Ref.</t>
         </is>
       </c>
-      <c r="N9" s="9" t="inlineStr">
+      <c r="N9" s="10" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="n">
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="B10" s="10" t="n"/>
-      <c r="C10" s="10" t="n"/>
-      <c r="D10" s="10" t="n"/>
-      <c r="E10" s="10" t="n"/>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-      <c r="H10" s="10" t="n"/>
-      <c r="I10" s="10" t="n"/>
-      <c r="J10" s="10" t="n"/>
-      <c r="K10" s="10" t="n"/>
-      <c r="L10" s="10" t="n"/>
-      <c r="M10" s="10" t="n"/>
-      <c r="N10" s="10" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="n">
+      <c r="B10" s="11" t="n"/>
+      <c r="C10" s="11" t="n"/>
+      <c r="D10" s="11" t="n"/>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="11" t="n"/>
+      <c r="I10" s="11" t="n"/>
+      <c r="J10" s="11" t="n"/>
+      <c r="K10" s="11" t="n"/>
+      <c r="L10" s="11" t="n"/>
+      <c r="M10" s="11" t="n"/>
+      <c r="N10" s="11" t="n"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="B11" s="11" t="n"/>
-      <c r="C11" s="11" t="n"/>
-      <c r="D11" s="11" t="n"/>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
-      <c r="H11" s="11" t="n"/>
-      <c r="I11" s="11" t="n"/>
-      <c r="J11" s="11" t="n"/>
-      <c r="K11" s="11" t="n"/>
-      <c r="L11" s="11" t="n"/>
-      <c r="M11" s="11" t="n"/>
-      <c r="N11" s="11" t="n"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="n">
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="12" t="n"/>
+      <c r="I11" s="12" t="n"/>
+      <c r="J11" s="12" t="n"/>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="12" t="n"/>
+      <c r="M11" s="12" t="n"/>
+      <c r="N11" s="12" t="n"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="11" t="n">
         <v>3</v>
       </c>
-      <c r="B12" s="10" t="n"/>
-      <c r="C12" s="10" t="n"/>
-      <c r="D12" s="10" t="n"/>
-      <c r="E12" s="10" t="n"/>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-      <c r="H12" s="10" t="n"/>
-      <c r="I12" s="10" t="n"/>
-      <c r="J12" s="10" t="n"/>
-      <c r="K12" s="10" t="n"/>
-      <c r="L12" s="10" t="n"/>
-      <c r="M12" s="10" t="n"/>
-      <c r="N12" s="10" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="11" t="n">
+      <c r="B12" s="11" t="n"/>
+      <c r="C12" s="11" t="n"/>
+      <c r="D12" s="11" t="n"/>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="11" t="n"/>
+      <c r="I12" s="11" t="n"/>
+      <c r="J12" s="11" t="n"/>
+      <c r="K12" s="11" t="n"/>
+      <c r="L12" s="11" t="n"/>
+      <c r="M12" s="11" t="n"/>
+      <c r="N12" s="11" t="n"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="12" t="n">
         <v>4</v>
       </c>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="11" t="n"/>
-      <c r="D13" s="11" t="n"/>
-      <c r="E13" s="11" t="n"/>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="11" t="n"/>
-      <c r="H13" s="11" t="n"/>
-      <c r="I13" s="11" t="n"/>
-      <c r="J13" s="11" t="n"/>
-      <c r="K13" s="11" t="n"/>
-      <c r="L13" s="11" t="n"/>
-      <c r="M13" s="11" t="n"/>
-      <c r="N13" s="11" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="10" t="n">
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="12" t="n"/>
+      <c r="I13" s="12" t="n"/>
+      <c r="J13" s="12" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="12" t="n"/>
+      <c r="M13" s="12" t="n"/>
+      <c r="N13" s="12" t="n"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="11" t="n">
         <v>5</v>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-      <c r="H14" s="10" t="n"/>
-      <c r="I14" s="10" t="n"/>
-      <c r="J14" s="10" t="n"/>
-      <c r="K14" s="10" t="n"/>
-      <c r="L14" s="10" t="n"/>
-      <c r="M14" s="10" t="n"/>
-      <c r="N14" s="10" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="n">
+      <c r="B14" s="11" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="11" t="n"/>
+      <c r="E14" s="11" t="n"/>
+      <c r="F14" s="11" t="n"/>
+      <c r="G14" s="11" t="n"/>
+      <c r="H14" s="11" t="n"/>
+      <c r="I14" s="11" t="n"/>
+      <c r="J14" s="11" t="n"/>
+      <c r="K14" s="11" t="n"/>
+      <c r="L14" s="11" t="n"/>
+      <c r="M14" s="11" t="n"/>
+      <c r="N14" s="11" t="n"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="12" t="n">
         <v>6</v>
       </c>
-      <c r="B15" s="11" t="n"/>
-      <c r="C15" s="11" t="n"/>
-      <c r="D15" s="11" t="n"/>
-      <c r="E15" s="11" t="n"/>
-      <c r="F15" s="11" t="n"/>
-      <c r="G15" s="11" t="n"/>
-      <c r="H15" s="11" t="n"/>
-      <c r="I15" s="11" t="n"/>
-      <c r="J15" s="11" t="n"/>
-      <c r="K15" s="11" t="n"/>
-      <c r="L15" s="11" t="n"/>
-      <c r="M15" s="11" t="n"/>
-      <c r="N15" s="11" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="10" t="n">
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="12" t="n"/>
+      <c r="I15" s="12" t="n"/>
+      <c r="J15" s="12" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="12" t="n"/>
+      <c r="M15" s="12" t="n"/>
+      <c r="N15" s="12" t="n"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="11" t="n">
         <v>7</v>
       </c>
-      <c r="B16" s="10" t="n"/>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-      <c r="H16" s="10" t="n"/>
-      <c r="I16" s="10" t="n"/>
-      <c r="J16" s="10" t="n"/>
-      <c r="K16" s="10" t="n"/>
-      <c r="L16" s="10" t="n"/>
-      <c r="M16" s="10" t="n"/>
-      <c r="N16" s="10" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="11" t="n">
+      <c r="B16" s="11" t="n"/>
+      <c r="C16" s="11" t="n"/>
+      <c r="D16" s="11" t="n"/>
+      <c r="E16" s="11" t="n"/>
+      <c r="F16" s="11" t="n"/>
+      <c r="G16" s="11" t="n"/>
+      <c r="H16" s="11" t="n"/>
+      <c r="I16" s="11" t="n"/>
+      <c r="J16" s="11" t="n"/>
+      <c r="K16" s="11" t="n"/>
+      <c r="L16" s="11" t="n"/>
+      <c r="M16" s="11" t="n"/>
+      <c r="N16" s="11" t="n"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="12" t="n">
         <v>8</v>
       </c>
-      <c r="B17" s="11" t="n"/>
-      <c r="C17" s="11" t="n"/>
-      <c r="D17" s="11" t="n"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
-      <c r="H17" s="11" t="n"/>
-      <c r="I17" s="11" t="n"/>
-      <c r="J17" s="11" t="n"/>
-      <c r="K17" s="11" t="n"/>
-      <c r="L17" s="11" t="n"/>
-      <c r="M17" s="11" t="n"/>
-      <c r="N17" s="11" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="10" t="n">
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="12" t="n"/>
+      <c r="I17" s="12" t="n"/>
+      <c r="J17" s="12" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="12" t="n"/>
+      <c r="M17" s="12" t="n"/>
+      <c r="N17" s="12" t="n"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="11" t="n">
         <v>9</v>
       </c>
-      <c r="B18" s="10" t="n"/>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-      <c r="H18" s="10" t="n"/>
-      <c r="I18" s="10" t="n"/>
-      <c r="J18" s="10" t="n"/>
-      <c r="K18" s="10" t="n"/>
-      <c r="L18" s="10" t="n"/>
-      <c r="M18" s="10" t="n"/>
-      <c r="N18" s="10" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="11" t="n">
+      <c r="B18" s="11" t="n"/>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="11" t="n"/>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="11" t="n"/>
+      <c r="I18" s="11" t="n"/>
+      <c r="J18" s="11" t="n"/>
+      <c r="K18" s="11" t="n"/>
+      <c r="L18" s="11" t="n"/>
+      <c r="M18" s="11" t="n"/>
+      <c r="N18" s="11" t="n"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="B19" s="11" t="n"/>
-      <c r="C19" s="11" t="n"/>
-      <c r="D19" s="11" t="n"/>
-      <c r="E19" s="11" t="n"/>
-      <c r="F19" s="11" t="n"/>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="11" t="n"/>
-      <c r="I19" s="11" t="n"/>
-      <c r="J19" s="11" t="n"/>
-      <c r="K19" s="11" t="n"/>
-      <c r="L19" s="11" t="n"/>
-      <c r="M19" s="11" t="n"/>
-      <c r="N19" s="11" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="10" t="n">
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="12" t="n"/>
+      <c r="J19" s="12" t="n"/>
+      <c r="K19" s="12" t="n"/>
+      <c r="L19" s="12" t="n"/>
+      <c r="M19" s="12" t="n"/>
+      <c r="N19" s="12" t="n"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="11" t="n">
         <v>11</v>
       </c>
-      <c r="B20" s="10" t="n"/>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-      <c r="H20" s="10" t="n"/>
-      <c r="I20" s="10" t="n"/>
-      <c r="J20" s="10" t="n"/>
-      <c r="K20" s="10" t="n"/>
-      <c r="L20" s="10" t="n"/>
-      <c r="M20" s="10" t="n"/>
-      <c r="N20" s="10" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="11" t="n">
+      <c r="B20" s="11" t="n"/>
+      <c r="C20" s="11" t="n"/>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="11" t="n"/>
+      <c r="G20" s="11" t="n"/>
+      <c r="H20" s="11" t="n"/>
+      <c r="I20" s="11" t="n"/>
+      <c r="J20" s="11" t="n"/>
+      <c r="K20" s="11" t="n"/>
+      <c r="L20" s="11" t="n"/>
+      <c r="M20" s="11" t="n"/>
+      <c r="N20" s="11" t="n"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="B21" s="11" t="n"/>
-      <c r="C21" s="11" t="n"/>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
-      <c r="F21" s="11" t="n"/>
-      <c r="G21" s="11" t="n"/>
-      <c r="H21" s="11" t="n"/>
-      <c r="I21" s="11" t="n"/>
-      <c r="J21" s="11" t="n"/>
-      <c r="K21" s="11" t="n"/>
-      <c r="L21" s="11" t="n"/>
-      <c r="M21" s="11" t="n"/>
-      <c r="N21" s="11" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="n">
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="12" t="n"/>
+      <c r="I21" s="12" t="n"/>
+      <c r="J21" s="12" t="n"/>
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="12" t="n"/>
+      <c r="M21" s="12" t="n"/>
+      <c r="N21" s="12" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="11" t="n">
         <v>13</v>
       </c>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-      <c r="H22" s="10" t="n"/>
-      <c r="I22" s="10" t="n"/>
-      <c r="J22" s="10" t="n"/>
-      <c r="K22" s="10" t="n"/>
-      <c r="L22" s="10" t="n"/>
-      <c r="M22" s="10" t="n"/>
-      <c r="N22" s="10" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="11" t="n">
+      <c r="B22" s="11" t="n"/>
+      <c r="C22" s="11" t="n"/>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
+      <c r="F22" s="11" t="n"/>
+      <c r="G22" s="11" t="n"/>
+      <c r="H22" s="11" t="n"/>
+      <c r="I22" s="11" t="n"/>
+      <c r="J22" s="11" t="n"/>
+      <c r="K22" s="11" t="n"/>
+      <c r="L22" s="11" t="n"/>
+      <c r="M22" s="11" t="n"/>
+      <c r="N22" s="11" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="12" t="n">
         <v>14</v>
       </c>
-      <c r="B23" s="11" t="n"/>
-      <c r="C23" s="11" t="n"/>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
-      <c r="F23" s="11" t="n"/>
-      <c r="G23" s="11" t="n"/>
-      <c r="H23" s="11" t="n"/>
-      <c r="I23" s="11" t="n"/>
-      <c r="J23" s="11" t="n"/>
-      <c r="K23" s="11" t="n"/>
-      <c r="L23" s="11" t="n"/>
-      <c r="M23" s="11" t="n"/>
-      <c r="N23" s="11" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="n">
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="12" t="n"/>
+      <c r="I23" s="12" t="n"/>
+      <c r="J23" s="12" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="12" t="n"/>
+      <c r="M23" s="12" t="n"/>
+      <c r="N23" s="12" t="n"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="11" t="n">
         <v>15</v>
       </c>
-      <c r="B24" s="10" t="n"/>
-      <c r="C24" s="10" t="n"/>
-      <c r="D24" s="10" t="n"/>
-      <c r="E24" s="10" t="n"/>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
-      <c r="H24" s="10" t="n"/>
-      <c r="I24" s="10" t="n"/>
-      <c r="J24" s="10" t="n"/>
-      <c r="K24" s="10" t="n"/>
-      <c r="L24" s="10" t="n"/>
-      <c r="M24" s="10" t="n"/>
-      <c r="N24" s="10" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="11" t="n">
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="11" t="n"/>
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
+      <c r="H24" s="11" t="n"/>
+      <c r="I24" s="11" t="n"/>
+      <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="n"/>
+      <c r="L24" s="11" t="n"/>
+      <c r="M24" s="11" t="n"/>
+      <c r="N24" s="11" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="12" t="n">
         <v>16</v>
       </c>
-      <c r="B25" s="11" t="n"/>
-      <c r="C25" s="11" t="n"/>
-      <c r="D25" s="11" t="n"/>
-      <c r="E25" s="11" t="n"/>
-      <c r="F25" s="11" t="n"/>
-      <c r="G25" s="11" t="n"/>
-      <c r="H25" s="11" t="n"/>
-      <c r="I25" s="11" t="n"/>
-      <c r="J25" s="11" t="n"/>
-      <c r="K25" s="11" t="n"/>
-      <c r="L25" s="11" t="n"/>
-      <c r="M25" s="11" t="n"/>
-      <c r="N25" s="11" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="n">
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="12" t="n"/>
+      <c r="I25" s="12" t="n"/>
+      <c r="J25" s="12" t="n"/>
+      <c r="K25" s="12" t="n"/>
+      <c r="L25" s="12" t="n"/>
+      <c r="M25" s="12" t="n"/>
+      <c r="N25" s="12" t="n"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="11" t="n">
         <v>17</v>
       </c>
-      <c r="B26" s="10" t="n"/>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
-      <c r="H26" s="10" t="n"/>
-      <c r="I26" s="10" t="n"/>
-      <c r="J26" s="10" t="n"/>
-      <c r="K26" s="10" t="n"/>
-      <c r="L26" s="10" t="n"/>
-      <c r="M26" s="10" t="n"/>
-      <c r="N26" s="10" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="11" t="n">
+      <c r="B26" s="11" t="n"/>
+      <c r="C26" s="11" t="n"/>
+      <c r="D26" s="11" t="n"/>
+      <c r="E26" s="11" t="n"/>
+      <c r="F26" s="11" t="n"/>
+      <c r="G26" s="11" t="n"/>
+      <c r="H26" s="11" t="n"/>
+      <c r="I26" s="11" t="n"/>
+      <c r="J26" s="11" t="n"/>
+      <c r="K26" s="11" t="n"/>
+      <c r="L26" s="11" t="n"/>
+      <c r="M26" s="11" t="n"/>
+      <c r="N26" s="11" t="n"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="12" t="n">
         <v>18</v>
       </c>
-      <c r="B27" s="11" t="n"/>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="11" t="n"/>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="11" t="n"/>
-      <c r="G27" s="11" t="n"/>
-      <c r="H27" s="11" t="n"/>
-      <c r="I27" s="11" t="n"/>
-      <c r="J27" s="11" t="n"/>
-      <c r="K27" s="11" t="n"/>
-      <c r="L27" s="11" t="n"/>
-      <c r="M27" s="11" t="n"/>
-      <c r="N27" s="11" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="10" t="n">
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="12" t="n"/>
+      <c r="I27" s="12" t="n"/>
+      <c r="J27" s="12" t="n"/>
+      <c r="K27" s="12" t="n"/>
+      <c r="L27" s="12" t="n"/>
+      <c r="M27" s="12" t="n"/>
+      <c r="N27" s="12" t="n"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="11" t="n">
         <v>19</v>
       </c>
-      <c r="B28" s="10" t="n"/>
-      <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
-      <c r="H28" s="10" t="n"/>
-      <c r="I28" s="10" t="n"/>
-      <c r="J28" s="10" t="n"/>
-      <c r="K28" s="10" t="n"/>
-      <c r="L28" s="10" t="n"/>
-      <c r="M28" s="10" t="n"/>
-      <c r="N28" s="10" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="11" t="n">
+      <c r="B28" s="11" t="n"/>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="11" t="n"/>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="11" t="n"/>
+      <c r="G28" s="11" t="n"/>
+      <c r="H28" s="11" t="n"/>
+      <c r="I28" s="11" t="n"/>
+      <c r="J28" s="11" t="n"/>
+      <c r="K28" s="11" t="n"/>
+      <c r="L28" s="11" t="n"/>
+      <c r="M28" s="11" t="n"/>
+      <c r="N28" s="11" t="n"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="12" t="n">
         <v>20</v>
       </c>
-      <c r="B29" s="11" t="n"/>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="11" t="n"/>
-      <c r="E29" s="11" t="n"/>
-      <c r="F29" s="11" t="n"/>
-      <c r="G29" s="11" t="n"/>
-      <c r="H29" s="11" t="n"/>
-      <c r="I29" s="11" t="n"/>
-      <c r="J29" s="11" t="n"/>
-      <c r="K29" s="11" t="n"/>
-      <c r="L29" s="11" t="n"/>
-      <c r="M29" s="11" t="n"/>
-      <c r="N29" s="11" t="n"/>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="12" t="n"/>
+      <c r="I29" s="12" t="n"/>
+      <c r="J29" s="12" t="n"/>
+      <c r="K29" s="12" t="n"/>
+      <c r="L29" s="12" t="n"/>
+      <c r="M29" s="12" t="n"/>
+      <c r="N29" s="12" t="n"/>
     </row>
     <row r="31" ht="3" customHeight="1">
       <c r="A31" s="5" t="n"/>
@@ -1119,25 +1144,25 @@
       <c r="M31" s="5" t="n"/>
       <c r="N31" s="5" t="n"/>
     </row>
-    <row r="32">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>PECH Group Holdings Ltd  |  Confidential  |  pechgroupholdings.tech  |  Technology &amp; Infrastructure Enablers for People</t>
-        </is>
-      </c>
-      <c r="B32" s="13" t="n"/>
-      <c r="C32" s="13" t="n"/>
-      <c r="D32" s="13" t="n"/>
-      <c r="E32" s="13" t="n"/>
-      <c r="F32" s="13" t="n"/>
-      <c r="G32" s="13" t="n"/>
-      <c r="H32" s="13" t="n"/>
-      <c r="I32" s="13" t="n"/>
-      <c r="J32" s="13" t="n"/>
-      <c r="K32" s="13" t="n"/>
-      <c r="L32" s="13" t="n"/>
-      <c r="M32" s="13" t="n"/>
-      <c r="N32" s="13" t="n"/>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="13" t="inlineStr">
+        <is>
+          <t>Confidential  |  pechgroupholdings.tech  |  Technology &amp; Infrastructure Enablers for People</t>
+        </is>
+      </c>
+      <c r="B32" s="7" t="n"/>
+      <c r="C32" s="7" t="n"/>
+      <c r="D32" s="7" t="n"/>
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="7" t="n"/>
+      <c r="H32" s="7" t="n"/>
+      <c r="I32" s="7" t="n"/>
+      <c r="J32" s="7" t="n"/>
+      <c r="K32" s="7" t="n"/>
+      <c r="L32" s="7" t="n"/>
+      <c r="M32" s="7" t="n"/>
+      <c r="N32" s="7" t="n"/>
     </row>
     <row r="33" ht="3" customHeight="1">
       <c r="A33" s="1" t="n"/>

</xml_diff>